<commit_message>
update img dashboard v2
</commit_message>
<xml_diff>
--- a/outputs/churn_backtest_nov.xlsx
+++ b/outputs/churn_backtest_nov.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="nov_backtest" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="nov_backtest" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -566,7 +566,7 @@
         <v>1</v>
       </c>
       <c r="O2" t="n">
-        <v>0.741677463054657</v>
+        <v>0.7415364980697632</v>
       </c>
       <c r="P2" t="n">
         <v>1</v>
@@ -622,19 +622,19 @@
         <v>1</v>
       </c>
       <c r="K3" t="n">
-        <v>0.5404380986990592</v>
+        <v>0.5404380986990589</v>
       </c>
       <c r="L3" t="n">
         <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>0.6367634286272592</v>
+        <v>0.6367634286272593</v>
       </c>
       <c r="N3" t="n">
         <v>1</v>
       </c>
       <c r="O3" t="n">
-        <v>0.5088237524032593</v>
+        <v>0.5088819265365601</v>
       </c>
       <c r="P3" t="n">
         <v>1</v>
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>0.6367634286272592</v>
+        <v>0.6367634286272593</v>
       </c>
       <c r="T3" t="n">
         <v>1</v>
@@ -702,7 +702,7 @@
         <v>1</v>
       </c>
       <c r="O4" t="n">
-        <v>0.6851392388343811</v>
+        <v>0.6851956248283386</v>
       </c>
       <c r="P4" t="n">
         <v>1</v>
@@ -758,19 +758,19 @@
         <v>2</v>
       </c>
       <c r="K5" t="n">
-        <v>0.02928779861824864</v>
+        <v>0.02928779861824868</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>0.2294097217862421</v>
+        <v>0.2294097217862422</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>0.06759648770093918</v>
+        <v>0.06750812381505966</v>
       </c>
       <c r="P5" t="n">
         <v>0</v>
@@ -784,7 +784,7 @@
         </is>
       </c>
       <c r="S5" t="n">
-        <v>0.2294097217862421</v>
+        <v>0.2294097217862422</v>
       </c>
       <c r="T5" t="n">
         <v>0</v>
@@ -832,13 +832,13 @@
         <v>1</v>
       </c>
       <c r="M6" t="n">
-        <v>0.6045709548864392</v>
+        <v>0.6045709548864393</v>
       </c>
       <c r="N6" t="n">
         <v>1</v>
       </c>
       <c r="O6" t="n">
-        <v>0.6209129691123962</v>
+        <v>0.6209686398506165</v>
       </c>
       <c r="P6" t="n">
         <v>1</v>
@@ -852,7 +852,7 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>0.6045709548864392</v>
+        <v>0.6045709548864393</v>
       </c>
       <c r="T6" t="n">
         <v>1</v>
@@ -894,7 +894,7 @@
         <v>1</v>
       </c>
       <c r="K7" t="n">
-        <v>0.6859289474551495</v>
+        <v>0.6859289474551494</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -906,7 +906,7 @@
         <v>1</v>
       </c>
       <c r="O7" t="n">
-        <v>0.6655395030975342</v>
+        <v>0.6655784249305725</v>
       </c>
       <c r="P7" t="n">
         <v>1</v>
@@ -974,7 +974,7 @@
         <v>0</v>
       </c>
       <c r="O8" t="n">
-        <v>0.1018329858779907</v>
+        <v>0.1017190590500832</v>
       </c>
       <c r="P8" t="n">
         <v>0</v>
@@ -1030,7 +1030,7 @@
         <v>1</v>
       </c>
       <c r="K9" t="n">
-        <v>0.6378200934827836</v>
+        <v>0.6378200934827835</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1042,7 +1042,7 @@
         <v>1</v>
       </c>
       <c r="O9" t="n">
-        <v>0.6688246726989746</v>
+        <v>0.6686413884162903</v>
       </c>
       <c r="P9" t="n">
         <v>1</v>
@@ -1110,7 +1110,7 @@
         <v>1</v>
       </c>
       <c r="O10" t="n">
-        <v>0.417546272277832</v>
+        <v>0.4176041483879089</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1166,7 +1166,7 @@
         <v>2</v>
       </c>
       <c r="K11" t="n">
-        <v>0.3635653034389554</v>
+        <v>0.3635653034389553</v>
       </c>
       <c r="L11" t="n">
         <v>1</v>
@@ -1178,7 +1178,7 @@
         <v>1</v>
       </c>
       <c r="O11" t="n">
-        <v>0.7048625946044922</v>
+        <v>0.7046977877616882</v>
       </c>
       <c r="P11" t="n">
         <v>1</v>
@@ -1240,13 +1240,13 @@
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>0.3382326892473237</v>
+        <v>0.3382326892473238</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
       </c>
       <c r="O12" t="n">
-        <v>0.1368114203214645</v>
+        <v>0.1366600841283798</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
@@ -1260,7 +1260,7 @@
         </is>
       </c>
       <c r="S12" t="n">
-        <v>0.3382326892473237</v>
+        <v>0.3382326892473238</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1314,7 +1314,7 @@
         <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>0.2859717309474945</v>
+        <v>0.2860417366027832</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
@@ -1382,7 +1382,7 @@
         <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>0.4101652503013611</v>
+        <v>0.4099863767623901</v>
       </c>
       <c r="P14" t="n">
         <v>0</v>
@@ -1444,13 +1444,13 @@
         <v>1</v>
       </c>
       <c r="M15" t="n">
-        <v>0.3622235677615618</v>
+        <v>0.3622235677615619</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
       </c>
       <c r="O15" t="n">
-        <v>0.3296981155872345</v>
+        <v>0.3294138312339783</v>
       </c>
       <c r="P15" t="n">
         <v>0</v>
@@ -1464,7 +1464,7 @@
         </is>
       </c>
       <c r="S15" t="n">
-        <v>0.3622235677615618</v>
+        <v>0.3622235677615619</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1506,19 +1506,19 @@
         <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>0.6941578605650018</v>
+        <v>0.6941578605650017</v>
       </c>
       <c r="L16" t="n">
         <v>1</v>
       </c>
       <c r="M16" t="n">
-        <v>0.6358206124351421</v>
+        <v>0.6358206124351422</v>
       </c>
       <c r="N16" t="n">
         <v>1</v>
       </c>
       <c r="O16" t="n">
-        <v>0.4673353135585785</v>
+        <v>0.4673746228218079</v>
       </c>
       <c r="P16" t="n">
         <v>0</v>
@@ -1532,7 +1532,7 @@
         </is>
       </c>
       <c r="S16" t="n">
-        <v>0.6358206124351421</v>
+        <v>0.6358206124351422</v>
       </c>
       <c r="T16" t="n">
         <v>1</v>
@@ -1586,7 +1586,7 @@
         <v>1</v>
       </c>
       <c r="O17" t="n">
-        <v>0.8218982815742493</v>
+        <v>0.821778416633606</v>
       </c>
       <c r="P17" t="n">
         <v>1</v>
@@ -1642,7 +1642,7 @@
         <v>2</v>
       </c>
       <c r="K18" t="n">
-        <v>0.0690564668608544</v>
+        <v>0.06905646686085437</v>
       </c>
       <c r="L18" t="n">
         <v>0</v>
@@ -1654,7 +1654,7 @@
         <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>0.1265901476144791</v>
+        <v>0.126627117395401</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1722,7 +1722,7 @@
         <v>1</v>
       </c>
       <c r="O19" t="n">
-        <v>0.5071833729743958</v>
+        <v>0.5072267055511475</v>
       </c>
       <c r="P19" t="n">
         <v>1</v>
@@ -1790,7 +1790,7 @@
         <v>1</v>
       </c>
       <c r="O20" t="n">
-        <v>0.6295484304428101</v>
+        <v>0.6296057105064392</v>
       </c>
       <c r="P20" t="n">
         <v>1</v>
@@ -1858,7 +1858,7 @@
         <v>1</v>
       </c>
       <c r="O21" t="n">
-        <v>0.7060428857803345</v>
+        <v>0.7058923840522766</v>
       </c>
       <c r="P21" t="n">
         <v>1</v>
@@ -1914,19 +1914,19 @@
         <v>2</v>
       </c>
       <c r="K22" t="n">
-        <v>0.03011706285142695</v>
+        <v>0.03011706285142694</v>
       </c>
       <c r="L22" t="n">
         <v>0</v>
       </c>
       <c r="M22" t="n">
-        <v>0.2629150889324888</v>
+        <v>0.2629150889324889</v>
       </c>
       <c r="N22" t="n">
         <v>0</v>
       </c>
       <c r="O22" t="n">
-        <v>0.1113569512963295</v>
+        <v>0.1112296804785728</v>
       </c>
       <c r="P22" t="n">
         <v>0</v>
@@ -1940,7 +1940,7 @@
         </is>
       </c>
       <c r="S22" t="n">
-        <v>0.2629150889324888</v>
+        <v>0.2629150889324889</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -1994,7 +1994,7 @@
         <v>0</v>
       </c>
       <c r="O23" t="n">
-        <v>0.07554208487272263</v>
+        <v>0.07545407861471176</v>
       </c>
       <c r="P23" t="n">
         <v>0</v>
@@ -2050,7 +2050,7 @@
         <v>1</v>
       </c>
       <c r="K24" t="n">
-        <v>0.4213038958718631</v>
+        <v>0.4213038958718632</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -2062,7 +2062,7 @@
         <v>0</v>
       </c>
       <c r="O24" t="n">
-        <v>0.3553758859634399</v>
+        <v>0.3552071750164032</v>
       </c>
       <c r="P24" t="n">
         <v>0</v>
@@ -2118,19 +2118,19 @@
         <v>2</v>
       </c>
       <c r="K25" t="n">
-        <v>0.02721815377643943</v>
+        <v>0.02721815377643945</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
       </c>
       <c r="M25" t="n">
-        <v>0.3015595783523888</v>
+        <v>0.3015595783523889</v>
       </c>
       <c r="N25" t="n">
         <v>0</v>
       </c>
       <c r="O25" t="n">
-        <v>0.2231060713529587</v>
+        <v>0.2228714525699615</v>
       </c>
       <c r="P25" t="n">
         <v>0</v>
@@ -2144,7 +2144,7 @@
         </is>
       </c>
       <c r="S25" t="n">
-        <v>0.3015595783523888</v>
+        <v>0.3015595783523889</v>
       </c>
       <c r="T25" t="n">
         <v>0</v>
@@ -2186,7 +2186,7 @@
         <v>1</v>
       </c>
       <c r="K26" t="n">
-        <v>0.7048000583119921</v>
+        <v>0.704800058311992</v>
       </c>
       <c r="L26" t="n">
         <v>1</v>
@@ -2198,7 +2198,7 @@
         <v>1</v>
       </c>
       <c r="O26" t="n">
-        <v>0.6449657678604126</v>
+        <v>0.6447794437408447</v>
       </c>
       <c r="P26" t="n">
         <v>1</v>
@@ -2260,13 +2260,13 @@
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>0.6709827451776977</v>
+        <v>0.6709827451776976</v>
       </c>
       <c r="N27" t="n">
         <v>1</v>
       </c>
       <c r="O27" t="n">
-        <v>0.7404813170433044</v>
+        <v>0.7405163645744324</v>
       </c>
       <c r="P27" t="n">
         <v>1</v>
@@ -2280,7 +2280,7 @@
         </is>
       </c>
       <c r="S27" t="n">
-        <v>0.6709827451776977</v>
+        <v>0.6709827451776976</v>
       </c>
       <c r="T27" t="n">
         <v>1</v>
@@ -2322,19 +2322,19 @@
         <v>2</v>
       </c>
       <c r="K28" t="n">
-        <v>0.1468061460712948</v>
+        <v>0.1468061460712947</v>
       </c>
       <c r="L28" t="n">
         <v>0</v>
       </c>
       <c r="M28" t="n">
-        <v>0.3162699288873393</v>
+        <v>0.3162699288873394</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>0.1285417824983597</v>
+        <v>0.1285749524831772</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2348,7 +2348,7 @@
         </is>
       </c>
       <c r="S28" t="n">
-        <v>0.3162699288873393</v>
+        <v>0.3162699288873394</v>
       </c>
       <c r="T28" t="n">
         <v>0</v>
@@ -2396,13 +2396,13 @@
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>0.503866743134488</v>
+        <v>0.5038667431344881</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>0.4318293035030365</v>
+        <v>0.4318923950195312</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2416,7 +2416,7 @@
         </is>
       </c>
       <c r="S29" t="n">
-        <v>0.503866743134488</v>
+        <v>0.5038667431344881</v>
       </c>
       <c r="T29" t="n">
         <v>0</v>
@@ -2464,13 +2464,13 @@
         <v>0</v>
       </c>
       <c r="M30" t="n">
-        <v>0.2447668548000008</v>
+        <v>0.2447668548000009</v>
       </c>
       <c r="N30" t="n">
         <v>0</v>
       </c>
       <c r="O30" t="n">
-        <v>0.07972943037748337</v>
+        <v>0.07962745428085327</v>
       </c>
       <c r="P30" t="n">
         <v>0</v>
@@ -2484,7 +2484,7 @@
         </is>
       </c>
       <c r="S30" t="n">
-        <v>0.2447668548000008</v>
+        <v>0.2447668548000009</v>
       </c>
       <c r="T30" t="n">
         <v>0</v>
@@ -2538,7 +2538,7 @@
         <v>0</v>
       </c>
       <c r="O31" t="n">
-        <v>0.1036505922675133</v>
+        <v>0.1035231128334999</v>
       </c>
       <c r="P31" t="n">
         <v>0</v>
@@ -2594,19 +2594,19 @@
         <v>2</v>
       </c>
       <c r="K32" t="n">
-        <v>0.07595664554669065</v>
+        <v>0.0759566455466907</v>
       </c>
       <c r="L32" t="n">
         <v>0</v>
       </c>
       <c r="M32" t="n">
-        <v>0.3072665218065284</v>
+        <v>0.3072665218065285</v>
       </c>
       <c r="N32" t="n">
         <v>0</v>
       </c>
       <c r="O32" t="n">
-        <v>0.1676826626062393</v>
+        <v>0.1675815582275391</v>
       </c>
       <c r="P32" t="n">
         <v>0</v>
@@ -2620,7 +2620,7 @@
         </is>
       </c>
       <c r="S32" t="n">
-        <v>0.3072665218065284</v>
+        <v>0.3072665218065285</v>
       </c>
       <c r="T32" t="n">
         <v>0</v>
@@ -2674,7 +2674,7 @@
         <v>1</v>
       </c>
       <c r="O33" t="n">
-        <v>0.6724907755851746</v>
+        <v>0.6725376844406128</v>
       </c>
       <c r="P33" t="n">
         <v>1</v>
@@ -2736,13 +2736,13 @@
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>0.6101401632634142</v>
+        <v>0.6101401632634144</v>
       </c>
       <c r="N34" t="n">
         <v>1</v>
       </c>
       <c r="O34" t="n">
-        <v>0.3859857320785522</v>
+        <v>0.3860337436199188</v>
       </c>
       <c r="P34" t="n">
         <v>0</v>
@@ -2756,7 +2756,7 @@
         </is>
       </c>
       <c r="S34" t="n">
-        <v>0.6101401632634142</v>
+        <v>0.6101401632634144</v>
       </c>
       <c r="T34" t="n">
         <v>1</v>
@@ -2798,19 +2798,19 @@
         <v>2</v>
       </c>
       <c r="K35" t="n">
-        <v>0.2199580005028357</v>
+        <v>0.2199580005028358</v>
       </c>
       <c r="L35" t="n">
         <v>0</v>
       </c>
       <c r="M35" t="n">
-        <v>0.3592110509005004</v>
+        <v>0.3592110509005005</v>
       </c>
       <c r="N35" t="n">
         <v>0</v>
       </c>
       <c r="O35" t="n">
-        <v>0.271728515625</v>
+        <v>0.2718000113964081</v>
       </c>
       <c r="P35" t="n">
         <v>0</v>
@@ -2824,7 +2824,7 @@
         </is>
       </c>
       <c r="S35" t="n">
-        <v>0.3592110509005004</v>
+        <v>0.3592110509005005</v>
       </c>
       <c r="T35" t="n">
         <v>0</v>
@@ -2878,7 +2878,7 @@
         <v>1</v>
       </c>
       <c r="O36" t="n">
-        <v>0.693145215511322</v>
+        <v>0.6932094693183899</v>
       </c>
       <c r="P36" t="n">
         <v>1</v>
@@ -2934,7 +2934,7 @@
         <v>1</v>
       </c>
       <c r="K37" t="n">
-        <v>0.6220452792898042</v>
+        <v>0.6220452792898039</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
@@ -2946,7 +2946,7 @@
         <v>1</v>
       </c>
       <c r="O37" t="n">
-        <v>0.6221215128898621</v>
+        <v>0.6221686601638794</v>
       </c>
       <c r="P37" t="n">
         <v>1</v>
@@ -3008,13 +3008,13 @@
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>0.5380230930245646</v>
+        <v>0.5380230930245647</v>
       </c>
       <c r="N38" t="n">
         <v>1</v>
       </c>
       <c r="O38" t="n">
-        <v>0.6656369566917419</v>
+        <v>0.6653367877006531</v>
       </c>
       <c r="P38" t="n">
         <v>1</v>
@@ -3028,7 +3028,7 @@
         </is>
       </c>
       <c r="S38" t="n">
-        <v>0.5380230930245646</v>
+        <v>0.5380230930245647</v>
       </c>
       <c r="T38" t="n">
         <v>1</v>
@@ -3076,13 +3076,13 @@
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>0.6448100606383225</v>
+        <v>0.6448100606383224</v>
       </c>
       <c r="N39" t="n">
         <v>1</v>
       </c>
       <c r="O39" t="n">
-        <v>0.6386719942092896</v>
+        <v>0.638716995716095</v>
       </c>
       <c r="P39" t="n">
         <v>1</v>
@@ -3096,7 +3096,7 @@
         </is>
       </c>
       <c r="S39" t="n">
-        <v>0.6448100606383225</v>
+        <v>0.6448100606383224</v>
       </c>
       <c r="T39" t="n">
         <v>1</v>
@@ -3138,7 +3138,7 @@
         <v>1</v>
       </c>
       <c r="K40" t="n">
-        <v>0.7135566972141864</v>
+        <v>0.7135566972141862</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
@@ -3150,7 +3150,7 @@
         <v>1</v>
       </c>
       <c r="O40" t="n">
-        <v>0.7429636120796204</v>
+        <v>0.7428136467933655</v>
       </c>
       <c r="P40" t="n">
         <v>1</v>
@@ -3206,7 +3206,7 @@
         <v>1</v>
       </c>
       <c r="K41" t="n">
-        <v>0.6097880126178662</v>
+        <v>0.6097880126178663</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
@@ -3218,7 +3218,7 @@
         <v>0</v>
       </c>
       <c r="O41" t="n">
-        <v>0.3697740435600281</v>
+        <v>0.3694527149200439</v>
       </c>
       <c r="P41" t="n">
         <v>0</v>
@@ -3274,7 +3274,7 @@
         <v>2</v>
       </c>
       <c r="K42" t="n">
-        <v>0.2196421557321498</v>
+        <v>0.2196421557321499</v>
       </c>
       <c r="L42" t="n">
         <v>0</v>
@@ -3286,7 +3286,7 @@
         <v>1</v>
       </c>
       <c r="O42" t="n">
-        <v>0.5766241550445557</v>
+        <v>0.5764317512512207</v>
       </c>
       <c r="P42" t="n">
         <v>1</v>
@@ -3354,7 +3354,7 @@
         <v>1</v>
       </c>
       <c r="O43" t="n">
-        <v>0.5165666341781616</v>
+        <v>0.5166337490081787</v>
       </c>
       <c r="P43" t="n">
         <v>1</v>
@@ -3416,13 +3416,13 @@
         <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>0.5494789628767093</v>
+        <v>0.5494789628767092</v>
       </c>
       <c r="N44" t="n">
         <v>1</v>
       </c>
       <c r="O44" t="n">
-        <v>0.5606684684753418</v>
+        <v>0.5604827404022217</v>
       </c>
       <c r="P44" t="n">
         <v>1</v>
@@ -3436,7 +3436,7 @@
         </is>
       </c>
       <c r="S44" t="n">
-        <v>0.5494789628767093</v>
+        <v>0.5494789628767092</v>
       </c>
       <c r="T44" t="n">
         <v>1</v>
@@ -3478,7 +3478,7 @@
         <v>1</v>
       </c>
       <c r="K45" t="n">
-        <v>0.5759313268434413</v>
+        <v>0.5759313268434411</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
@@ -3490,7 +3490,7 @@
         <v>1</v>
       </c>
       <c r="O45" t="n">
-        <v>0.4395902156829834</v>
+        <v>0.4396484196186066</v>
       </c>
       <c r="P45" t="n">
         <v>0</v>
@@ -3546,7 +3546,7 @@
         <v>1</v>
       </c>
       <c r="K46" t="n">
-        <v>0.7478880162339678</v>
+        <v>0.7478880162339679</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
@@ -3558,7 +3558,7 @@
         <v>1</v>
       </c>
       <c r="O46" t="n">
-        <v>0.6339532732963562</v>
+        <v>0.6337743401527405</v>
       </c>
       <c r="P46" t="n">
         <v>1</v>
@@ -3614,19 +3614,19 @@
         <v>1</v>
       </c>
       <c r="K47" t="n">
-        <v>0.6218641363224204</v>
+        <v>0.6218641363224203</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>0.5756172643541407</v>
+        <v>0.5756172643541408</v>
       </c>
       <c r="N47" t="n">
         <v>1</v>
       </c>
       <c r="O47" t="n">
-        <v>0.6678728461265564</v>
+        <v>0.6677060127258301</v>
       </c>
       <c r="P47" t="n">
         <v>1</v>
@@ -3640,7 +3640,7 @@
         </is>
       </c>
       <c r="S47" t="n">
-        <v>0.5756172643541407</v>
+        <v>0.5756172643541408</v>
       </c>
       <c r="T47" t="n">
         <v>1</v>
@@ -3694,7 +3694,7 @@
         <v>0</v>
       </c>
       <c r="O48" t="n">
-        <v>0.1887191534042358</v>
+        <v>0.1885051280260086</v>
       </c>
       <c r="P48" t="n">
         <v>0</v>
@@ -3750,19 +3750,19 @@
         <v>1</v>
       </c>
       <c r="K49" t="n">
-        <v>0.1580574327173853</v>
+        <v>0.1580574327173852</v>
       </c>
       <c r="L49" t="n">
         <v>0</v>
       </c>
       <c r="M49" t="n">
-        <v>0.3590320235800054</v>
+        <v>0.3590320235800055</v>
       </c>
       <c r="N49" t="n">
         <v>0</v>
       </c>
       <c r="O49" t="n">
-        <v>0.3061262369155884</v>
+        <v>0.3059724569320679</v>
       </c>
       <c r="P49" t="n">
         <v>0</v>
@@ -3776,7 +3776,7 @@
         </is>
       </c>
       <c r="S49" t="n">
-        <v>0.3590320235800054</v>
+        <v>0.3590320235800055</v>
       </c>
       <c r="T49" t="n">
         <v>0</v>
@@ -3818,19 +3818,19 @@
         <v>1</v>
       </c>
       <c r="K50" t="n">
-        <v>0.2916220326989725</v>
+        <v>0.2916220326989726</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>0.2321042154707682</v>
+        <v>0.2321042154707683</v>
       </c>
       <c r="N50" t="n">
         <v>0</v>
       </c>
       <c r="O50" t="n">
-        <v>0.1383258253335953</v>
+        <v>0.1381778866052628</v>
       </c>
       <c r="P50" t="n">
         <v>0</v>
@@ -3844,7 +3844,7 @@
         </is>
       </c>
       <c r="S50" t="n">
-        <v>0.2321042154707682</v>
+        <v>0.2321042154707683</v>
       </c>
       <c r="T50" t="n">
         <v>0</v>
@@ -3886,19 +3886,19 @@
         <v>1</v>
       </c>
       <c r="K51" t="n">
-        <v>0.3453689785143254</v>
+        <v>0.3453689785143252</v>
       </c>
       <c r="L51" t="n">
         <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>0.4377215812946882</v>
+        <v>0.4377215812946884</v>
       </c>
       <c r="N51" t="n">
         <v>0</v>
       </c>
       <c r="O51" t="n">
-        <v>0.4883025884628296</v>
+        <v>0.4883766770362854</v>
       </c>
       <c r="P51" t="n">
         <v>0</v>
@@ -3912,7 +3912,7 @@
         </is>
       </c>
       <c r="S51" t="n">
-        <v>0.4377215812946882</v>
+        <v>0.4377215812946884</v>
       </c>
       <c r="T51" t="n">
         <v>0</v>
@@ -3954,19 +3954,19 @@
         <v>1</v>
       </c>
       <c r="K52" t="n">
-        <v>0.8113303985151958</v>
+        <v>0.8113303985151959</v>
       </c>
       <c r="L52" t="n">
         <v>1</v>
       </c>
       <c r="M52" t="n">
-        <v>0.6291554471372914</v>
+        <v>0.6291554471372915</v>
       </c>
       <c r="N52" t="n">
         <v>1</v>
       </c>
       <c r="O52" t="n">
-        <v>0.7781243324279785</v>
+        <v>0.7779948115348816</v>
       </c>
       <c r="P52" t="n">
         <v>1</v>
@@ -3980,7 +3980,7 @@
         </is>
       </c>
       <c r="S52" t="n">
-        <v>0.6291554471372914</v>
+        <v>0.6291554471372915</v>
       </c>
       <c r="T52" t="n">
         <v>1</v>
@@ -4028,13 +4028,13 @@
         <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>0.6940082584015861</v>
+        <v>0.6940082584015862</v>
       </c>
       <c r="N53" t="n">
         <v>1</v>
       </c>
       <c r="O53" t="n">
-        <v>0.8803350329399109</v>
+        <v>0.8802516460418701</v>
       </c>
       <c r="P53" t="n">
         <v>1</v>
@@ -4048,7 +4048,7 @@
         </is>
       </c>
       <c r="S53" t="n">
-        <v>0.6940082584015861</v>
+        <v>0.6940082584015862</v>
       </c>
       <c r="T53" t="n">
         <v>1</v>
@@ -4090,7 +4090,7 @@
         <v>2</v>
       </c>
       <c r="K54" t="n">
-        <v>0.08293916248098258</v>
+        <v>0.08293916248098263</v>
       </c>
       <c r="L54" t="n">
         <v>0</v>
@@ -4102,7 +4102,7 @@
         <v>0</v>
       </c>
       <c r="O54" t="n">
-        <v>0.1095863506197929</v>
+        <v>0.1094645708799362</v>
       </c>
       <c r="P54" t="n">
         <v>0</v>
@@ -4164,13 +4164,13 @@
         <v>0</v>
       </c>
       <c r="M55" t="n">
-        <v>0.3232702567338976</v>
+        <v>0.3232702567338977</v>
       </c>
       <c r="N55" t="n">
         <v>0</v>
       </c>
       <c r="O55" t="n">
-        <v>0.2464539706707001</v>
+        <v>0.2462216466665268</v>
       </c>
       <c r="P55" t="n">
         <v>0</v>
@@ -4184,7 +4184,7 @@
         </is>
       </c>
       <c r="S55" t="n">
-        <v>0.3232702567338976</v>
+        <v>0.3232702567338977</v>
       </c>
       <c r="T55" t="n">
         <v>0</v>
@@ -4226,7 +4226,7 @@
         <v>1</v>
       </c>
       <c r="K56" t="n">
-        <v>0.5226128785090526</v>
+        <v>0.5226128785090527</v>
       </c>
       <c r="L56" t="n">
         <v>1</v>
@@ -4238,7 +4238,7 @@
         <v>0</v>
       </c>
       <c r="O56" t="n">
-        <v>0.3866357207298279</v>
+        <v>0.3867148756980896</v>
       </c>
       <c r="P56" t="n">
         <v>0</v>
@@ -4294,19 +4294,19 @@
         <v>1</v>
       </c>
       <c r="K57" t="n">
-        <v>0.554673444850831</v>
+        <v>0.5546734448508308</v>
       </c>
       <c r="L57" t="n">
         <v>1</v>
       </c>
       <c r="M57" t="n">
-        <v>0.536649265235726</v>
+        <v>0.5366492652357261</v>
       </c>
       <c r="N57" t="n">
         <v>0</v>
       </c>
       <c r="O57" t="n">
-        <v>0.6494291424751282</v>
+        <v>0.6492584943771362</v>
       </c>
       <c r="P57" t="n">
         <v>1</v>
@@ -4320,7 +4320,7 @@
         </is>
       </c>
       <c r="S57" t="n">
-        <v>0.536649265235726</v>
+        <v>0.5366492652357261</v>
       </c>
       <c r="T57" t="n">
         <v>0</v>
@@ -4362,19 +4362,19 @@
         <v>1</v>
       </c>
       <c r="K58" t="n">
-        <v>0.7245430386124319</v>
+        <v>0.7245430386124317</v>
       </c>
       <c r="L58" t="n">
         <v>1</v>
       </c>
       <c r="M58" t="n">
-        <v>0.597345909423583</v>
+        <v>0.5973459094235831</v>
       </c>
       <c r="N58" t="n">
         <v>1</v>
       </c>
       <c r="O58" t="n">
-        <v>0.6719260811805725</v>
+        <v>0.6719743013381958</v>
       </c>
       <c r="P58" t="n">
         <v>1</v>
@@ -4388,7 +4388,7 @@
         </is>
       </c>
       <c r="S58" t="n">
-        <v>0.597345909423583</v>
+        <v>0.5973459094235831</v>
       </c>
       <c r="T58" t="n">
         <v>1</v>
@@ -4436,13 +4436,13 @@
         <v>0</v>
       </c>
       <c r="M59" t="n">
-        <v>0.3001811331956283</v>
+        <v>0.3001811331956284</v>
       </c>
       <c r="N59" t="n">
         <v>0</v>
       </c>
       <c r="O59" t="n">
-        <v>0.1777811944484711</v>
+        <v>0.1776766031980515</v>
       </c>
       <c r="P59" t="n">
         <v>0</v>
@@ -4456,7 +4456,7 @@
         </is>
       </c>
       <c r="S59" t="n">
-        <v>0.3001811331956283</v>
+        <v>0.3001811331956284</v>
       </c>
       <c r="T59" t="n">
         <v>0</v>
@@ -4498,7 +4498,7 @@
         <v>2</v>
       </c>
       <c r="K60" t="n">
-        <v>0.072999373007306</v>
+        <v>0.07299937300730602</v>
       </c>
       <c r="L60" t="n">
         <v>0</v>
@@ -4510,7 +4510,7 @@
         <v>0</v>
       </c>
       <c r="O60" t="n">
-        <v>0.06659500300884247</v>
+        <v>0.06650993973016739</v>
       </c>
       <c r="P60" t="n">
         <v>0</v>
@@ -4566,19 +4566,19 @@
         <v>1</v>
       </c>
       <c r="K61" t="n">
-        <v>0.2210842128899617</v>
+        <v>0.2210842128899616</v>
       </c>
       <c r="L61" t="n">
         <v>0</v>
       </c>
       <c r="M61" t="n">
-        <v>0.3200344463091621</v>
+        <v>0.3200344463091622</v>
       </c>
       <c r="N61" t="n">
         <v>0</v>
       </c>
       <c r="O61" t="n">
-        <v>0.1611592322587967</v>
+        <v>0.1609701961278915</v>
       </c>
       <c r="P61" t="n">
         <v>0</v>
@@ -4592,7 +4592,7 @@
         </is>
       </c>
       <c r="S61" t="n">
-        <v>0.3200344463091621</v>
+        <v>0.3200344463091622</v>
       </c>
       <c r="T61" t="n">
         <v>0</v>
@@ -4640,13 +4640,13 @@
         <v>1</v>
       </c>
       <c r="M62" t="n">
-        <v>0.6811203018080579</v>
+        <v>0.681120301808058</v>
       </c>
       <c r="N62" t="n">
         <v>1</v>
       </c>
       <c r="O62" t="n">
-        <v>0.8496155738830566</v>
+        <v>0.8495165705680847</v>
       </c>
       <c r="P62" t="n">
         <v>1</v>
@@ -4660,7 +4660,7 @@
         </is>
       </c>
       <c r="S62" t="n">
-        <v>0.6811203018080579</v>
+        <v>0.681120301808058</v>
       </c>
       <c r="T62" t="n">
         <v>1</v>
@@ -4702,19 +4702,19 @@
         <v>2</v>
       </c>
       <c r="K63" t="n">
-        <v>0.04471127073766586</v>
+        <v>0.0447112707376659</v>
       </c>
       <c r="L63" t="n">
         <v>0</v>
       </c>
       <c r="M63" t="n">
-        <v>0.3037136939603213</v>
+        <v>0.3037136939603214</v>
       </c>
       <c r="N63" t="n">
         <v>0</v>
       </c>
       <c r="O63" t="n">
-        <v>0.238298624753952</v>
+        <v>0.2381696850061417</v>
       </c>
       <c r="P63" t="n">
         <v>0</v>
@@ -4728,7 +4728,7 @@
         </is>
       </c>
       <c r="S63" t="n">
-        <v>0.3037136939603213</v>
+        <v>0.3037136939603214</v>
       </c>
       <c r="T63" t="n">
         <v>0</v>
@@ -4770,7 +4770,7 @@
         <v>2</v>
       </c>
       <c r="K64" t="n">
-        <v>0.07410719475006745</v>
+        <v>0.07410719475006743</v>
       </c>
       <c r="L64" t="n">
         <v>0</v>
@@ -4782,7 +4782,7 @@
         <v>0</v>
       </c>
       <c r="O64" t="n">
-        <v>0.2223509103059769</v>
+        <v>0.2222245782613754</v>
       </c>
       <c r="P64" t="n">
         <v>0</v>
@@ -4838,7 +4838,7 @@
         <v>1</v>
       </c>
       <c r="K65" t="n">
-        <v>0.5447179597338058</v>
+        <v>0.5447179597338057</v>
       </c>
       <c r="L65" t="n">
         <v>1</v>
@@ -4850,7 +4850,7 @@
         <v>0</v>
       </c>
       <c r="O65" t="n">
-        <v>0.4152809977531433</v>
+        <v>0.4153427481651306</v>
       </c>
       <c r="P65" t="n">
         <v>0</v>
@@ -4918,7 +4918,7 @@
         <v>1</v>
       </c>
       <c r="O66" t="n">
-        <v>0.6639152765274048</v>
+        <v>0.6639729738235474</v>
       </c>
       <c r="P66" t="n">
         <v>1</v>
@@ -4986,7 +4986,7 @@
         <v>1</v>
       </c>
       <c r="O67" t="n">
-        <v>0.417546272277832</v>
+        <v>0.4176041483879089</v>
       </c>
       <c r="P67" t="n">
         <v>0</v>
@@ -5048,13 +5048,13 @@
         <v>0</v>
       </c>
       <c r="M68" t="n">
-        <v>0.3466550066729814</v>
+        <v>0.3466550066729815</v>
       </c>
       <c r="N68" t="n">
         <v>0</v>
       </c>
       <c r="O68" t="n">
-        <v>0.1700439602136612</v>
+        <v>0.1698506623506546</v>
       </c>
       <c r="P68" t="n">
         <v>0</v>
@@ -5068,7 +5068,7 @@
         </is>
       </c>
       <c r="S68" t="n">
-        <v>0.3466550066729814</v>
+        <v>0.3466550066729815</v>
       </c>
       <c r="T68" t="n">
         <v>0</v>
@@ -5110,19 +5110,19 @@
         <v>2</v>
       </c>
       <c r="K69" t="n">
-        <v>0.1700903666614106</v>
+        <v>0.1700903666614105</v>
       </c>
       <c r="L69" t="n">
         <v>0</v>
       </c>
       <c r="M69" t="n">
-        <v>0.3860881601178373</v>
+        <v>0.3860881601178374</v>
       </c>
       <c r="N69" t="n">
         <v>0</v>
       </c>
       <c r="O69" t="n">
-        <v>0.2267075926065445</v>
+        <v>0.2267573773860931</v>
       </c>
       <c r="P69" t="n">
         <v>0</v>
@@ -5136,7 +5136,7 @@
         </is>
       </c>
       <c r="S69" t="n">
-        <v>0.3860881601178373</v>
+        <v>0.3860881601178374</v>
       </c>
       <c r="T69" t="n">
         <v>0</v>
@@ -5190,7 +5190,7 @@
         <v>1</v>
       </c>
       <c r="O70" t="n">
-        <v>0.4393084943294525</v>
+        <v>0.4393643140792847</v>
       </c>
       <c r="P70" t="n">
         <v>0</v>
@@ -5246,7 +5246,7 @@
         <v>1</v>
       </c>
       <c r="K71" t="n">
-        <v>0.3883375887158521</v>
+        <v>0.3883375887158522</v>
       </c>
       <c r="L71" t="n">
         <v>1</v>
@@ -5258,7 +5258,7 @@
         <v>0</v>
       </c>
       <c r="O71" t="n">
-        <v>0.2872646152973175</v>
+        <v>0.287007212638855</v>
       </c>
       <c r="P71" t="n">
         <v>0</v>
@@ -5326,7 +5326,7 @@
         <v>1</v>
       </c>
       <c r="O72" t="n">
-        <v>0.8156031966209412</v>
+        <v>0.8154833316802979</v>
       </c>
       <c r="P72" t="n">
         <v>1</v>
@@ -5394,7 +5394,7 @@
         <v>0</v>
       </c>
       <c r="O73" t="n">
-        <v>0.2092132419347763</v>
+        <v>0.2090000808238983</v>
       </c>
       <c r="P73" t="n">
         <v>0</v>
@@ -5450,19 +5450,19 @@
         <v>1</v>
       </c>
       <c r="K74" t="n">
-        <v>0.5934452453812562</v>
+        <v>0.593445245381256</v>
       </c>
       <c r="L74" t="n">
         <v>1</v>
       </c>
       <c r="M74" t="n">
-        <v>0.6200458254208792</v>
+        <v>0.620045825420879</v>
       </c>
       <c r="N74" t="n">
         <v>1</v>
       </c>
       <c r="O74" t="n">
-        <v>0.5256881713867188</v>
+        <v>0.5257365107536316</v>
       </c>
       <c r="P74" t="n">
         <v>1</v>
@@ -5476,7 +5476,7 @@
         </is>
       </c>
       <c r="S74" t="n">
-        <v>0.6200458254208792</v>
+        <v>0.620045825420879</v>
       </c>
       <c r="T74" t="n">
         <v>1</v>
@@ -5518,7 +5518,7 @@
         <v>1</v>
       </c>
       <c r="K75" t="n">
-        <v>0.4249081159529328</v>
+        <v>0.4249081159529327</v>
       </c>
       <c r="L75" t="n">
         <v>1</v>
@@ -5530,7 +5530,7 @@
         <v>1</v>
       </c>
       <c r="O75" t="n">
-        <v>0.6678728461265564</v>
+        <v>0.6677060127258301</v>
       </c>
       <c r="P75" t="n">
         <v>1</v>
@@ -5598,7 +5598,7 @@
         <v>1</v>
       </c>
       <c r="O76" t="n">
-        <v>0.6678728461265564</v>
+        <v>0.6677060127258301</v>
       </c>
       <c r="P76" t="n">
         <v>1</v>
@@ -5654,19 +5654,19 @@
         <v>2</v>
       </c>
       <c r="K77" t="n">
-        <v>0.08960441433645033</v>
+        <v>0.08960441433645031</v>
       </c>
       <c r="L77" t="n">
         <v>0</v>
       </c>
       <c r="M77" t="n">
-        <v>0.2506083155240453</v>
+        <v>0.2506083155240454</v>
       </c>
       <c r="N77" t="n">
         <v>0</v>
       </c>
       <c r="O77" t="n">
-        <v>0.1118556931614876</v>
+        <v>0.1118879243731499</v>
       </c>
       <c r="P77" t="n">
         <v>0</v>
@@ -5680,7 +5680,7 @@
         </is>
       </c>
       <c r="S77" t="n">
-        <v>0.2506083155240453</v>
+        <v>0.2506083155240454</v>
       </c>
       <c r="T77" t="n">
         <v>0</v>
@@ -5722,7 +5722,7 @@
         <v>2</v>
       </c>
       <c r="K78" t="n">
-        <v>0.08812956978485949</v>
+        <v>0.08812956978485952</v>
       </c>
       <c r="L78" t="n">
         <v>0</v>
@@ -5734,7 +5734,7 @@
         <v>0</v>
       </c>
       <c r="O78" t="n">
-        <v>0.09578245878219604</v>
+        <v>0.09567438066005707</v>
       </c>
       <c r="P78" t="n">
         <v>0</v>
@@ -5790,19 +5790,19 @@
         <v>1</v>
       </c>
       <c r="K79" t="n">
-        <v>0.6687309197067508</v>
+        <v>0.6687309197067506</v>
       </c>
       <c r="L79" t="n">
         <v>1</v>
       </c>
       <c r="M79" t="n">
-        <v>0.6575505544735362</v>
+        <v>0.6575505544735363</v>
       </c>
       <c r="N79" t="n">
         <v>1</v>
       </c>
       <c r="O79" t="n">
-        <v>0.7326358556747437</v>
+        <v>0.7324828505516052</v>
       </c>
       <c r="P79" t="n">
         <v>1</v>
@@ -5816,7 +5816,7 @@
         </is>
       </c>
       <c r="S79" t="n">
-        <v>0.6575505544735362</v>
+        <v>0.6575505544735363</v>
       </c>
       <c r="T79" t="n">
         <v>1</v>
@@ -5870,7 +5870,7 @@
         <v>1</v>
       </c>
       <c r="O80" t="n">
-        <v>0.7575616836547852</v>
+        <v>0.7574167847633362</v>
       </c>
       <c r="P80" t="n">
         <v>1</v>
@@ -5926,7 +5926,7 @@
         <v>1</v>
       </c>
       <c r="K81" t="n">
-        <v>0.4752506538752163</v>
+        <v>0.4752506538752164</v>
       </c>
       <c r="L81" t="n">
         <v>1</v>
@@ -5938,7 +5938,7 @@
         <v>0</v>
       </c>
       <c r="O81" t="n">
-        <v>0.5161136984825134</v>
+        <v>0.5159271955490112</v>
       </c>
       <c r="P81" t="n">
         <v>1</v>
@@ -6006,7 +6006,7 @@
         <v>0</v>
       </c>
       <c r="O82" t="n">
-        <v>0.5161136984825134</v>
+        <v>0.5159271955490112</v>
       </c>
       <c r="P82" t="n">
         <v>1</v>
@@ -6062,19 +6062,19 @@
         <v>2</v>
       </c>
       <c r="K83" t="n">
-        <v>0.029174318254807</v>
+        <v>0.02917431825480702</v>
       </c>
       <c r="L83" t="n">
         <v>0</v>
       </c>
       <c r="M83" t="n">
-        <v>0.2309909973145979</v>
+        <v>0.230990997314598</v>
       </c>
       <c r="N83" t="n">
         <v>0</v>
       </c>
       <c r="O83" t="n">
-        <v>0.07077173888683319</v>
+        <v>0.07067949324846268</v>
       </c>
       <c r="P83" t="n">
         <v>0</v>
@@ -6088,7 +6088,7 @@
         </is>
       </c>
       <c r="S83" t="n">
-        <v>0.2309909973145979</v>
+        <v>0.230990997314598</v>
       </c>
       <c r="T83" t="n">
         <v>0</v>
@@ -6130,7 +6130,7 @@
         <v>1</v>
       </c>
       <c r="K84" t="n">
-        <v>0.6219651712341808</v>
+        <v>0.6219651712341807</v>
       </c>
       <c r="L84" t="n">
         <v>1</v>
@@ -6142,7 +6142,7 @@
         <v>1</v>
       </c>
       <c r="O84" t="n">
-        <v>0.6342344284057617</v>
+        <v>0.6340445876121521</v>
       </c>
       <c r="P84" t="n">
         <v>1</v>
@@ -6210,7 +6210,7 @@
         <v>0</v>
       </c>
       <c r="O85" t="n">
-        <v>0.1723193228244781</v>
+        <v>0.1721321642398834</v>
       </c>
       <c r="P85" t="n">
         <v>0</v>
@@ -6266,7 +6266,7 @@
         <v>2</v>
       </c>
       <c r="K86" t="n">
-        <v>0.04403814237939359</v>
+        <v>0.04403814237939357</v>
       </c>
       <c r="L86" t="n">
         <v>0</v>
@@ -6278,7 +6278,7 @@
         <v>0</v>
       </c>
       <c r="O86" t="n">
-        <v>0.1027147173881531</v>
+        <v>0.1026003286242485</v>
       </c>
       <c r="P86" t="n">
         <v>0</v>
@@ -6334,7 +6334,7 @@
         <v>1</v>
       </c>
       <c r="K87" t="n">
-        <v>0.5030464183449719</v>
+        <v>0.503046418344972</v>
       </c>
       <c r="L87" t="n">
         <v>1</v>
@@ -6346,7 +6346,7 @@
         <v>0</v>
       </c>
       <c r="O87" t="n">
-        <v>0.5161136984825134</v>
+        <v>0.5159271955490112</v>
       </c>
       <c r="P87" t="n">
         <v>1</v>
@@ -6402,7 +6402,7 @@
         <v>1</v>
       </c>
       <c r="K88" t="n">
-        <v>0.6504761534368602</v>
+        <v>0.6504761534368598</v>
       </c>
       <c r="L88" t="n">
         <v>1</v>
@@ -6414,7 +6414,7 @@
         <v>1</v>
       </c>
       <c r="O88" t="n">
-        <v>0.7844348549842834</v>
+        <v>0.7843023538589478</v>
       </c>
       <c r="P88" t="n">
         <v>1</v>
@@ -6470,7 +6470,7 @@
         <v>1</v>
       </c>
       <c r="K89" t="n">
-        <v>0.7502766600537616</v>
+        <v>0.7502766600537614</v>
       </c>
       <c r="L89" t="n">
         <v>1</v>
@@ -6482,7 +6482,7 @@
         <v>1</v>
       </c>
       <c r="O89" t="n">
-        <v>0.8156031966209412</v>
+        <v>0.8154833316802979</v>
       </c>
       <c r="P89" t="n">
         <v>1</v>
@@ -6538,7 +6538,7 @@
         <v>2</v>
       </c>
       <c r="K90" t="n">
-        <v>0.08274041285165611</v>
+        <v>0.08274041285165608</v>
       </c>
       <c r="L90" t="n">
         <v>0</v>
@@ -6550,7 +6550,7 @@
         <v>0</v>
       </c>
       <c r="O90" t="n">
-        <v>0.1142941638827324</v>
+        <v>0.1143270805478096</v>
       </c>
       <c r="P90" t="n">
         <v>0</v>
@@ -6606,7 +6606,7 @@
         <v>1</v>
       </c>
       <c r="K91" t="n">
-        <v>0.44306086205502</v>
+        <v>0.4430608620550196</v>
       </c>
       <c r="L91" t="n">
         <v>1</v>
@@ -6618,7 +6618,7 @@
         <v>1</v>
       </c>
       <c r="O91" t="n">
-        <v>0.7108497023582458</v>
+        <v>0.7106878161430359</v>
       </c>
       <c r="P91" t="n">
         <v>1</v>
@@ -6686,7 +6686,7 @@
         <v>0</v>
       </c>
       <c r="O92" t="n">
-        <v>0.4273605942726135</v>
+        <v>0.4271753430366516</v>
       </c>
       <c r="P92" t="n">
         <v>0</v>
@@ -6754,7 +6754,7 @@
         <v>0</v>
       </c>
       <c r="O93" t="n">
-        <v>0.3446571528911591</v>
+        <v>0.3443673849105835</v>
       </c>
       <c r="P93" t="n">
         <v>0</v>
@@ -6810,7 +6810,7 @@
         <v>2</v>
       </c>
       <c r="K94" t="n">
-        <v>0.02632118107931865</v>
+        <v>0.02632118107931866</v>
       </c>
       <c r="L94" t="n">
         <v>0</v>
@@ -6822,7 +6822,7 @@
         <v>0</v>
       </c>
       <c r="O94" t="n">
-        <v>0.06965292990207672</v>
+        <v>0.06957115232944489</v>
       </c>
       <c r="P94" t="n">
         <v>0</v>
@@ -6878,7 +6878,7 @@
         <v>1</v>
       </c>
       <c r="K95" t="n">
-        <v>0.3587747004754496</v>
+        <v>0.3587747004754492</v>
       </c>
       <c r="L95" t="n">
         <v>1</v>
@@ -6890,7 +6890,7 @@
         <v>1</v>
       </c>
       <c r="O95" t="n">
-        <v>0.602936327457428</v>
+        <v>0.6029759645462036</v>
       </c>
       <c r="P95" t="n">
         <v>1</v>
@@ -6958,7 +6958,7 @@
         <v>0</v>
       </c>
       <c r="O96" t="n">
-        <v>0.5466433763504028</v>
+        <v>0.5464599132537842</v>
       </c>
       <c r="P96" t="n">
         <v>1</v>
@@ -7026,7 +7026,7 @@
         <v>0</v>
       </c>
       <c r="O97" t="n">
-        <v>0.4152809977531433</v>
+        <v>0.4153427481651306</v>
       </c>
       <c r="P97" t="n">
         <v>0</v>
@@ -7094,7 +7094,7 @@
         <v>0</v>
       </c>
       <c r="O98" t="n">
-        <v>0.2026976197957993</v>
+        <v>0.2024914026260376</v>
       </c>
       <c r="P98" t="n">
         <v>0</v>
@@ -7156,13 +7156,13 @@
         <v>0</v>
       </c>
       <c r="M99" t="n">
-        <v>0.4486768939935179</v>
+        <v>0.448676893993518</v>
       </c>
       <c r="N99" t="n">
         <v>0</v>
       </c>
       <c r="O99" t="n">
-        <v>0.5065165758132935</v>
+        <v>0.5063453316688538</v>
       </c>
       <c r="P99" t="n">
         <v>0</v>
@@ -7176,7 +7176,7 @@
         </is>
       </c>
       <c r="S99" t="n">
-        <v>0.4486768939935179</v>
+        <v>0.448676893993518</v>
       </c>
       <c r="T99" t="n">
         <v>0</v>
@@ -7218,7 +7218,7 @@
         <v>1</v>
       </c>
       <c r="K100" t="n">
-        <v>0.8076943961524565</v>
+        <v>0.8076943961524563</v>
       </c>
       <c r="L100" t="n">
         <v>1</v>
@@ -7230,7 +7230,7 @@
         <v>1</v>
       </c>
       <c r="O100" t="n">
-        <v>0.8076958060264587</v>
+        <v>0.8075693249702454</v>
       </c>
       <c r="P100" t="n">
         <v>1</v>
@@ -7286,19 +7286,19 @@
         <v>2</v>
       </c>
       <c r="K101" t="n">
-        <v>0.08033144752825953</v>
+        <v>0.08033144752825958</v>
       </c>
       <c r="L101" t="n">
         <v>0</v>
       </c>
       <c r="M101" t="n">
-        <v>0.2892291027265077</v>
+        <v>0.2892291027265078</v>
       </c>
       <c r="N101" t="n">
         <v>0</v>
       </c>
       <c r="O101" t="n">
-        <v>0.1252296715974808</v>
+        <v>0.1250892132520676</v>
       </c>
       <c r="P101" t="n">
         <v>0</v>
@@ -7312,7 +7312,7 @@
         </is>
       </c>
       <c r="S101" t="n">
-        <v>0.2892291027265077</v>
+        <v>0.2892291027265078</v>
       </c>
       <c r="T101" t="n">
         <v>0</v>
@@ -7366,7 +7366,7 @@
         <v>0</v>
       </c>
       <c r="O102" t="n">
-        <v>0.1121964380145073</v>
+        <v>0.1120730191469193</v>
       </c>
       <c r="P102" t="n">
         <v>0</v>
@@ -7428,13 +7428,13 @@
         <v>0</v>
       </c>
       <c r="M103" t="n">
-        <v>0.3470682991377733</v>
+        <v>0.3470682991377734</v>
       </c>
       <c r="N103" t="n">
         <v>0</v>
       </c>
       <c r="O103" t="n">
-        <v>0.2204602062702179</v>
+        <v>0.2202489078044891</v>
       </c>
       <c r="P103" t="n">
         <v>0</v>
@@ -7448,7 +7448,7 @@
         </is>
       </c>
       <c r="S103" t="n">
-        <v>0.3470682991377733</v>
+        <v>0.3470682991377734</v>
       </c>
       <c r="T103" t="n">
         <v>0</v>
@@ -7502,7 +7502,7 @@
         <v>1</v>
       </c>
       <c r="O104" t="n">
-        <v>0.8046423196792603</v>
+        <v>0.8045149445533752</v>
       </c>
       <c r="P104" t="n">
         <v>1</v>
@@ -7570,7 +7570,7 @@
         <v>1</v>
       </c>
       <c r="O105" t="n">
-        <v>0.5748085975646973</v>
+        <v>0.5748621225357056</v>
       </c>
       <c r="P105" t="n">
         <v>1</v>
@@ -7626,7 +7626,7 @@
         <v>2</v>
       </c>
       <c r="K106" t="n">
-        <v>0.5033517136585008</v>
+        <v>0.503351713658501</v>
       </c>
       <c r="L106" t="n">
         <v>1</v>
@@ -7638,7 +7638,7 @@
         <v>1</v>
       </c>
       <c r="O106" t="n">
-        <v>0.7194433808326721</v>
+        <v>0.7192884683609009</v>
       </c>
       <c r="P106" t="n">
         <v>1</v>
@@ -7694,7 +7694,7 @@
         <v>2</v>
       </c>
       <c r="K107" t="n">
-        <v>0.3562613046919635</v>
+        <v>0.3562613046919637</v>
       </c>
       <c r="L107" t="n">
         <v>1</v>
@@ -7706,7 +7706,7 @@
         <v>0</v>
       </c>
       <c r="O107" t="n">
-        <v>0.4322016537189484</v>
+        <v>0.4322694838047028</v>
       </c>
       <c r="P107" t="n">
         <v>0</v>
@@ -7762,7 +7762,7 @@
         <v>2</v>
       </c>
       <c r="K108" t="n">
-        <v>0.08674530524835296</v>
+        <v>0.08674530524835299</v>
       </c>
       <c r="L108" t="n">
         <v>0</v>
@@ -7774,7 +7774,7 @@
         <v>0</v>
       </c>
       <c r="O108" t="n">
-        <v>0.1625785231590271</v>
+        <v>0.1624801605939865</v>
       </c>
       <c r="P108" t="n">
         <v>0</v>
@@ -7842,7 +7842,7 @@
         <v>0</v>
       </c>
       <c r="O109" t="n">
-        <v>0.315593808889389</v>
+        <v>0.3153217136859894</v>
       </c>
       <c r="P109" t="n">
         <v>0</v>
@@ -7898,19 +7898,19 @@
         <v>1</v>
       </c>
       <c r="K110" t="n">
-        <v>0.5128235130014225</v>
+        <v>0.5128235130014224</v>
       </c>
       <c r="L110" t="n">
         <v>1</v>
       </c>
       <c r="M110" t="n">
-        <v>0.5917938224366993</v>
+        <v>0.5917938224366994</v>
       </c>
       <c r="N110" t="n">
         <v>1</v>
       </c>
       <c r="O110" t="n">
-        <v>0.6863157749176025</v>
+        <v>0.6863510012626648</v>
       </c>
       <c r="P110" t="n">
         <v>1</v>
@@ -7924,7 +7924,7 @@
         </is>
       </c>
       <c r="S110" t="n">
-        <v>0.5917938224366993</v>
+        <v>0.5917938224366994</v>
       </c>
       <c r="T110" t="n">
         <v>1</v>
@@ -7966,7 +7966,7 @@
         <v>1</v>
       </c>
       <c r="K111" t="n">
-        <v>0.4575939554886375</v>
+        <v>0.4575939554886373</v>
       </c>
       <c r="L111" t="n">
         <v>1</v>
@@ -7978,7 +7978,7 @@
         <v>0</v>
       </c>
       <c r="O111" t="n">
-        <v>0.4114724397659302</v>
+        <v>0.411129355430603</v>
       </c>
       <c r="P111" t="n">
         <v>0</v>
@@ -8040,13 +8040,13 @@
         <v>1</v>
       </c>
       <c r="M112" t="n">
-        <v>0.5855820951969285</v>
+        <v>0.5855820951969287</v>
       </c>
       <c r="N112" t="n">
         <v>1</v>
       </c>
       <c r="O112" t="n">
-        <v>0.3642977774143219</v>
+        <v>0.3643390834331512</v>
       </c>
       <c r="P112" t="n">
         <v>0</v>
@@ -8060,7 +8060,7 @@
         </is>
       </c>
       <c r="S112" t="n">
-        <v>0.5855820951969285</v>
+        <v>0.5855820951969287</v>
       </c>
       <c r="T112" t="n">
         <v>1</v>
@@ -8102,7 +8102,7 @@
         <v>1</v>
       </c>
       <c r="K113" t="n">
-        <v>0.1946495715155855</v>
+        <v>0.1946495715155853</v>
       </c>
       <c r="L113" t="n">
         <v>0</v>
@@ -8114,7 +8114,7 @@
         <v>0</v>
       </c>
       <c r="O113" t="n">
-        <v>0.4130109846591949</v>
+        <v>0.4130677878856659</v>
       </c>
       <c r="P113" t="n">
         <v>0</v>
@@ -8170,7 +8170,7 @@
         <v>2</v>
       </c>
       <c r="K114" t="n">
-        <v>0.08029692636325284</v>
+        <v>0.08029692636325286</v>
       </c>
       <c r="L114" t="n">
         <v>0</v>
@@ -8182,7 +8182,7 @@
         <v>0</v>
       </c>
       <c r="O114" t="n">
-        <v>0.2462727427482605</v>
+        <v>0.246341273188591</v>
       </c>
       <c r="P114" t="n">
         <v>0</v>
@@ -8238,7 +8238,7 @@
         <v>1</v>
       </c>
       <c r="K115" t="n">
-        <v>0.7323705774307545</v>
+        <v>0.7323705774307544</v>
       </c>
       <c r="L115" t="n">
         <v>1</v>
@@ -8250,7 +8250,7 @@
         <v>1</v>
       </c>
       <c r="O115" t="n">
-        <v>0.5706232786178589</v>
+        <v>0.570677638053894</v>
       </c>
       <c r="P115" t="n">
         <v>1</v>
@@ -8306,7 +8306,7 @@
         <v>1</v>
       </c>
       <c r="K116" t="n">
-        <v>0.5146518412402382</v>
+        <v>0.5146518412402379</v>
       </c>
       <c r="L116" t="n">
         <v>1</v>
@@ -8318,7 +8318,7 @@
         <v>1</v>
       </c>
       <c r="O116" t="n">
-        <v>0.7110204696655273</v>
+        <v>0.7110581994056702</v>
       </c>
       <c r="P116" t="n">
         <v>1</v>
@@ -8374,7 +8374,7 @@
         <v>1</v>
       </c>
       <c r="K117" t="n">
-        <v>0.6089171174756097</v>
+        <v>0.6089171174756095</v>
       </c>
       <c r="L117" t="n">
         <v>1</v>
@@ -8386,7 +8386,7 @@
         <v>1</v>
       </c>
       <c r="O117" t="n">
-        <v>0.7203801870346069</v>
+        <v>0.7202158570289612</v>
       </c>
       <c r="P117" t="n">
         <v>1</v>

</xml_diff>